<commit_message>
refactor(report): generalize Excel template rendering
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/reports/monthly_labor_cost_list.xlsx
+++ b/backend/src/main/resources/reports/monthly_labor_cost_list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026.4" sheetId="81" r:id="R7df1226294b845aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026.4" sheetId="81" r:id="Ra61e2cdce5464e10"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -467,16 +467,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F1" s="7" t="str">
-        <x:v>${targetYear}年</x:v>
+        <x:v>${target_month:yyyy}年</x:v>
       </x:c>
       <x:c r="G1" s="9" t="str">
-        <x:v>${targetMonthValue}月分</x:v>
+        <x:v>${target_month:M}月分</x:v>
       </x:c>
       <x:c r="H1" s="17" t="str">
-        <x:v>${paymentMonth}/${paymentDay}支払</x:v>
+        <x:v>${payment_date:M}/${payment_date:d}支払</x:v>
       </x:c>
       <x:c r="AA1" t="str">
-        <x:v>${companyName}</x:v>
+        <x:v>${company_name}</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -572,47 +572,95 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="14"/>
-      <x:c r="B4" s="1"/>
-      <x:c r="C4" s="1"/>
-      <x:c r="D4" s="5"/>
-      <x:c r="E4" s="5"/>
-      <x:c r="F4" s="2"/>
-      <x:c r="G4" s="1"/>
-      <x:c r="H4" s="8"/>
-      <x:c r="I4" s="8"/>
-      <x:c r="J4" s="8"/>
-      <x:c r="K4" s="8"/>
+      <x:c r="A4" s="14" t="str">
+        <x:v>${row.employee_name}</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="str">
+        <x:v>${row.work_day_count}</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>${row.paid_leave_days}</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>${row.overtime_hours}</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>${row.night_work_hours}</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
+        <x:v>${row.basic_salary}</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>${row.overtime_pay_amount}</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>${row.night_pay_amount}</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>${row.driver_allowance_amount}</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
+        <x:v>${row.other_allowance_amount}</x:v>
+      </x:c>
+      <x:c r="K4" s="8" t="str">
+        <x:v>${row.business_trip_allowance_amount}</x:v>
+      </x:c>
       <x:c r="L4" s="21" t="str">
-        <x:f>IF($A4="","",SUM(F4:K4))</x:f>
-      </x:c>
-      <x:c r="M4" s="2"/>
-      <x:c r="N4" s="2"/>
-      <x:c r="O4" s="2"/>
-      <x:c r="P4" s="1"/>
+        <x:f>IF(OR($A4="",LEFT($A4,2)="${"),"",SUM(F4:K4))</x:f>
+      </x:c>
+      <x:c r="M4" s="2" t="str">
+        <x:v>${row.health_insurance}</x:v>
+      </x:c>
+      <x:c r="N4" s="2" t="str">
+        <x:v>${row.child_care_contribution}</x:v>
+      </x:c>
+      <x:c r="O4" s="2" t="str">
+        <x:v>${row.pension_insurance}</x:v>
+      </x:c>
+      <x:c r="P4" s="1" t="str">
+        <x:v>${row.employment_insurance}</x:v>
+      </x:c>
       <x:c r="Q4" s="2" t="str">
-        <x:f>IF($A4="","",SUM(M4:P4))</x:f>
+        <x:f>IF(OR($A4="",LEFT($A4,2)="${"),"",SUM(M4:P4))</x:f>
       </x:c>
       <x:c r="R4" s="2" t="str">
-        <x:f>IF($A4="","",L4-Q4)</x:f>
-      </x:c>
-      <x:c r="S4" s="21"/>
-      <x:c r="T4" s="2"/>
-      <x:c r="U4" s="8"/>
-      <x:c r="V4" s="8"/>
-      <x:c r="W4" s="8"/>
-      <x:c r="X4" s="8"/>
-      <x:c r="Y4" s="8"/>
+        <x:f>IF(OR($A4="",LEFT($A4,2)="${"),"",L4-Q4)</x:f>
+      </x:c>
+      <x:c r="S4" s="21" t="str">
+        <x:v>${row.income_tax}</x:v>
+      </x:c>
+      <x:c r="T4" s="2" t="str">
+        <x:v>${row.year_end_adjustment_amount}</x:v>
+      </x:c>
+      <x:c r="U4" s="8" t="str">
+        <x:v>${row.resident_tax}</x:v>
+      </x:c>
+      <x:c r="V4" s="8" t="str">
+        <x:v>${row.dormitory_fee_amount}</x:v>
+      </x:c>
+      <x:c r="W4" s="8" t="str">
+        <x:v>${row.mobile_rental_amount}</x:v>
+      </x:c>
+      <x:c r="X4" s="8" t="str">
+        <x:v>${row.wifi_fee_amount}</x:v>
+      </x:c>
+      <x:c r="Y4" s="8" t="str">
+        <x:v>${row.other_deduction_amount}</x:v>
+      </x:c>
       <x:c r="Z4" s="2" t="str">
-        <x:f>IF($A4="","",Q4+SUM(S4:Y4))</x:f>
+        <x:f>IF(OR($A4="",LEFT($A4,2)="${"),"",Q4+SUM(S4:Y4))</x:f>
       </x:c>
       <x:c r="AA4" s="2" t="str">
-        <x:f t="shared" ref="AA4:AA34" si="0">IF($A4="","",L4-Z4)</x:f>
-      </x:c>
-      <x:c r="AB4" s="1"/>
-      <x:c r="AC4" s="1"/>
+        <x:f t="shared" ref="AA4:AA34" si="0">IF(OR($A4="",LEFT($A4,2)="${"),"",L4-Z4)</x:f>
+      </x:c>
+      <x:c r="AB4" s="1" t="str">
+        <x:v>${row.advance_payment_amount}</x:v>
+      </x:c>
+      <x:c r="AC4" s="1" t="str">
+        <x:v>${row.saving_amount}</x:v>
+      </x:c>
       <x:c r="AD4" s="2" t="str">
-        <x:f>IF($A4="","",AA4-AB4-AC4)</x:f>
+        <x:f>IF(OR($A4="",LEFT($A4,2)="${"),"",AA4-AB4-AC4)</x:f>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>